<commit_message>
feat: show all epic features on roadmap hover tooltip
- Add epic_features column to store concatenated feature names per epic

- Populate epic_features during feature aggregation in roadmap_engine.py

- Display the feature list in charts.py Gantt tooltip instead of the epic name
</commit_message>
<xml_diff>
--- a/Backlog_Roadmap_2026.xlsx
+++ b/Backlog_Roadmap_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Consultor Noorden\Desktop\planning-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A541FFC9-54AD-464E-8152-FBB0FF2E6478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858D3C0E-6270-46C7-94DE-212C6DEA8FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,10 +42,41 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={5E7ADAE3-BFAF-4354-AE7C-4DA203F90938}</author>
+    <author>tc={C17263A4-E425-444C-BF97-70B1448F129A}</author>
+    <author>tc={4ACDD4B6-EB3F-4684-99D5-3EA6906C96CE}</author>
     <author>tc={5050488C-96D1-43A8-9998-3148830ABB2C}</author>
   </authors>
   <commentList>
-    <comment ref="C53" authorId="0" shapeId="0" xr:uid="{5050488C-96D1-43A8-9998-3148830ABB2C}">
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{5E7ADAE3-BFAF-4354-AE7C-4DA203F90938}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Eu subiria um pouco de prioridade (talvez 2) os épicos de sistematização porque eles podem ajudar na conformidade e no tempo de gerar as MFs. No frontend alguns filtros básicos já podem ser feitos para garantir menos problemas de ingestão ou dados errados.
+De todo modo esses desenvolvimentos tem um pouco menos de competição pelo tipo de recurso que utiliza, e devem ser feitos no futuro mais próximo
+Responder:
+    Concordo. Subi aqui a prioridade. Temos que avaliar porque temos uma sequência grande de homologações travadas já, mas acho que vale o push para o time de negócio.</t>
+      </text>
+    </comment>
+    <comment ref="C13" authorId="1" shapeId="0" xr:uid="{C17263A4-E425-444C-BF97-70B1448F129A}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Acredito que esse item por estar quente e afetar algumas respostas na visão de prontidão, podem ser mais prioritário no OTM2 que aquela questão de bandas na na função objetivo que ficou com prioridade 1. Eu as inverteria</t>
+      </text>
+    </comment>
+    <comment ref="C32" authorId="2" shapeId="0" xr:uid="{4ACDD4B6-EB3F-4684-99D5-3EA6906C96CE}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Eu entendi o ponto das features de monitoramente estejam a frente das de produtização que são 100% técnicas, porque elas trazem valor pro time de negócio.
+Eu só levaria em conta o risco de demorar a produtização técnica e isso poder ficar muito pra frente e ter problemas de orçamento ano que vem. Mas do ponto de vista de negócios, estou de acordo com a ordem</t>
+      </text>
+    </comment>
+    <comment ref="C53" authorId="3" shapeId="0" xr:uid="{5050488C-96D1-43A8-9998-3148830ABB2C}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -96,6 +127,120 @@
     <t>Mês sugerido</t>
   </si>
   <si>
+    <t>Produtização</t>
+  </si>
+  <si>
+    <t>Integração</t>
+  </si>
+  <si>
+    <t>Integração com SAP/Datalake (Para extrair automaticamente ZPS80)</t>
+  </si>
+  <si>
+    <t>Backlog Priorizado</t>
+  </si>
+  <si>
+    <t>Prontidão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestão de Processo </t>
+  </si>
+  <si>
+    <t>Olhar o longo prazo avaliando otimizador 2</t>
+  </si>
+  <si>
+    <t>Should Cost</t>
+  </si>
+  <si>
+    <t>Visibilidade de indicadores Shoud Cost</t>
+  </si>
+  <si>
+    <t>Criar output executivo replicando premissas da calculadora do Negocia+ (Suprimentos)</t>
+  </si>
+  <si>
+    <t>Realizar a Integração automatica com o LECOM</t>
+  </si>
+  <si>
+    <t>Melhorar Modelo Matemático OTM2</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixo] Introduzir bandas de custo na função objetivo</t>
+  </si>
+  <si>
+    <t>Backlog Parting Lote-BCG</t>
+  </si>
+  <si>
+    <t>Visibilidade e Acompanhamento de indicadores relacionados à prodidão</t>
+  </si>
+  <si>
+    <t>Mensurar o impacto da implementação da prorrogação</t>
+  </si>
+  <si>
+    <t>Conformidade</t>
+  </si>
+  <si>
+    <t>Melhorar Modelo Matemático OTM1</t>
+  </si>
+  <si>
+    <t>Criar Flag para priorização de pex criticos</t>
+  </si>
+  <si>
+    <t>Novo</t>
+  </si>
+  <si>
+    <t>Migração para ambiente de produção</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixo] Permitir rodar o Otimizador 2 com alvo fixo de kms de prontidão por período, sem depender do Otimizador 1</t>
+  </si>
+  <si>
+    <t>Automatizar indicadores no output dos planos gerados nas rodadas de otimização</t>
+  </si>
+  <si>
+    <t>Sistematização</t>
+  </si>
+  <si>
+    <t>Sistematização dos dados de RDO(Relatório diarios de obras)</t>
+  </si>
+  <si>
+    <t>Sistematização das informações de assentamentos</t>
+  </si>
+  <si>
+    <t>Sistematização das informações de arquetipos</t>
+  </si>
+  <si>
+    <t>Sistematização das informações de construcão</t>
+  </si>
+  <si>
+    <t>Exibição de indicadores executivos</t>
+  </si>
+  <si>
+    <t>Considerar trabalho aos Fins de semana</t>
+  </si>
+  <si>
+    <t>Avaliar incorporação de dados de autorização para trabalhos noturnos e aos fins de semana</t>
+  </si>
+  <si>
+    <t>Monitoramento</t>
+  </si>
+  <si>
+    <t>Executar a Pipeline de consistências antes da otimização</t>
+  </si>
+  <si>
+    <t>[OTM2] Feature mais de uma regra de inicio de projeto por municipio</t>
+  </si>
+  <si>
+    <t>[GATE 2] Calcular prontidão por contratada e região (Novo Filtro)</t>
+  </si>
+  <si>
+    <t>Criar 4 relatórios com dados para suportar decisões de prontidão</t>
+  </si>
+  <si>
+    <t>[Melhoria][Média] Criar uma lista de exceções para o Otimizador 2</t>
+  </si>
+  <si>
+    <t>Melhorar relatório de erros da ingestão</t>
+  </si>
+  <si>
     <t>Aderência</t>
   </si>
   <si>
@@ -105,67 +250,76 @@
     <t>Disponibilizar para o time de negócio um dashboard de Aderencia</t>
   </si>
   <si>
-    <t>Backlog Priorizado</t>
-  </si>
-  <si>
-    <t>Conformidade</t>
-  </si>
-  <si>
-    <t>Melhorar Modelo Matemático OTM1</t>
-  </si>
-  <si>
-    <t>Considerar trabalho aos Fins de semana</t>
-  </si>
-  <si>
-    <t>Avaliar incorporação de dados de autorização para trabalhos noturnos e aos fins de semana</t>
+    <t>Alteração no Otimizador 2 considerando os projetos Plano B</t>
+  </si>
+  <si>
+    <t>Simulador de Should Cost</t>
+  </si>
+  <si>
+    <t>Funcionalidade para simulações de cenários de Should Cost</t>
   </si>
   <si>
     <t>[Melhoria][Baixa] Flexibilizar datas de construção sugeridas pelo Otimizador 1 com penalização (restrições soft)</t>
   </si>
   <si>
-    <t>Backlog Parting Lote-BCG</t>
-  </si>
-  <si>
-    <t>Criar Flag para priorização de pex criticos</t>
-  </si>
-  <si>
-    <t>Novo</t>
-  </si>
-  <si>
-    <t>Produtização</t>
-  </si>
-  <si>
-    <t>Integração</t>
-  </si>
-  <si>
-    <t>Integração Service Now</t>
-  </si>
-  <si>
-    <t>Integração com SAP/Datalake (Para extrair automaticamente ZPS80)</t>
-  </si>
-  <si>
-    <t>Realizar a Integração automatica com o LECOM</t>
-  </si>
-  <si>
-    <t>Migração para ambiente de produção</t>
+    <t xml:space="preserve">Criar ferramenta visual de comparação de should cost entre os planos </t>
+  </si>
+  <si>
+    <t>Painel de acompanhamento dos indicadores técnicos de performance do modelo (Gap, runtime)</t>
+  </si>
+  <si>
+    <t>Expansão de escopo</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixo +] Adicionar escopo de vala aberta / loteamento</t>
+  </si>
+  <si>
+    <t>Elaborar relatório de erros da otimização</t>
+  </si>
+  <si>
+    <t>[Melhoria][Médio] Validar expectativas não cumpridas entre execuções automaticamente</t>
+  </si>
+  <si>
+    <t>Visualizações adicionais no produto</t>
+  </si>
+  <si>
+    <t>Criar uma gestão visual do acompanhamento da MF</t>
+  </si>
+  <si>
+    <t>[Melhoria][Media] Identificar automaticamente gargalos por semana, região ou fase</t>
+  </si>
+  <si>
+    <t>ADF - Repositório de engenharia de dados</t>
+  </si>
+  <si>
+    <t>Repositório do front-end</t>
+  </si>
+  <si>
+    <t>Migrar banco de dados do front-end</t>
+  </si>
+  <si>
+    <t>Jobs e workflows no Databricks</t>
+  </si>
+  <si>
+    <t>Migrar servidores que executam a aplicação do front-end (serviços do back e do front)</t>
+  </si>
+  <si>
+    <t>Processo de CI/CD</t>
+  </si>
+  <si>
+    <t>Tabelas no Databricks</t>
+  </si>
+  <si>
+    <t>Analisar os 600 projetos alocados na MF de Outubro</t>
   </si>
   <si>
     <t>Remover débito técnico de mapeamento de capacidade dos municípios que está direto no código</t>
   </si>
   <si>
-    <t>Arquivos no Sharepoint</t>
-  </si>
-  <si>
-    <t>ADF - Repositório de engenharia de dados</t>
-  </si>
-  <si>
-    <t>Repositório do front-end</t>
-  </si>
-  <si>
-    <t>Migrar servidores que executam a aplicação do front-end (serviços do back e do front)</t>
-  </si>
-  <si>
-    <t>Migrar banco de dados do front-end</t>
+    <t>Repositório de ciência de dados (Tatubo)</t>
+  </si>
+  <si>
+    <t>Flags na interface gráfica para consideração das excessões (individualmente) para facilitar não atualizar os inputs</t>
   </si>
   <si>
     <t>Integração entre ambientes
@@ -173,148 +327,25 @@
 ii. Comunicação entre sistemas para tráfego de dados (Servidor-Databricks)</t>
   </si>
   <si>
+    <t>Integração Service Now</t>
+  </si>
+  <si>
+    <t>Mapear os impactos da descontinuidade da GP (Ex: cadastros, plano vigente)</t>
+  </si>
+  <si>
+    <t>Criar ambiente para armazenar e tagear dados dos cenários simulados (inputs e outputs)</t>
+  </si>
+  <si>
+    <t>Débito técnico de desenvolvimentos hardcoded</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixo] Permitir rodar subconjuntos dos dados via filtro manual para ingestão</t>
+  </si>
+  <si>
     <t>Documentações</t>
   </si>
   <si>
-    <t>Processo de CI/CD</t>
-  </si>
-  <si>
-    <t>Tabelas no Databricks</t>
-  </si>
-  <si>
-    <t>Jobs e workflows no Databricks</t>
-  </si>
-  <si>
-    <t>Repositório de ciência de dados (Tatubo)</t>
-  </si>
-  <si>
-    <t>Analisar os 600 projetos alocados na MF de Outubro</t>
-  </si>
-  <si>
-    <t>[Melhoria][Baixo] Permitir rodar o Otimizador 2 com alvo fixo de kms de prontidão por período, sem depender do Otimizador 1</t>
-  </si>
-  <si>
-    <t>[Melhoria][Baixo] Permitir rodar subconjuntos dos dados via filtro manual para ingestão</t>
-  </si>
-  <si>
-    <t>Criar ambiente para armazenar e tagear dados dos cenários simulados (inputs e outputs)</t>
-  </si>
-  <si>
-    <t>Mapear os impactos da descontinuidade da GP (Ex: cadastros, plano vigente)</t>
-  </si>
-  <si>
-    <t>Flags na interface gráfica para consideração das excessões (individualmente) para facilitar não atualizar os inputs</t>
-  </si>
-  <si>
-    <t>Débito técnico de desenvolvimentos hardcoded</t>
-  </si>
-  <si>
-    <t>Monitoramento</t>
-  </si>
-  <si>
-    <t>Melhorar relatório de erros da ingestão</t>
-  </si>
-  <si>
-    <t>Executar a Pipeline de consistências antes da otmização</t>
-  </si>
-  <si>
-    <t>[Melhoria][Médio] Validar expectativas não cumpridas entre execuções automaticamente</t>
-  </si>
-  <si>
-    <t>Painel de acompanhamento dos indicadores técnicos de performance do modelo (Gap, runtime)</t>
-  </si>
-  <si>
-    <t>Elaborar relatório de erros da otimização</t>
-  </si>
-  <si>
-    <t>Sistematização</t>
-  </si>
-  <si>
-    <t>Sistematização dos dados de RDO(Relatório diarios de obras)</t>
-  </si>
-  <si>
-    <t>Sistematização das informações de assentamentos</t>
-  </si>
-  <si>
-    <t>Sistematização das informações de arquetipos</t>
-  </si>
-  <si>
-    <t>Sistematização das informações de construcão</t>
-  </si>
-  <si>
-    <t>Visualizações adicionais no produto</t>
-  </si>
-  <si>
-    <t>Criar uma gestão visual do acompanhamento da MF</t>
-  </si>
-  <si>
-    <t>Prontidão</t>
-  </si>
-  <si>
-    <t>Melhorar Modelo Matemático OTM2</t>
-  </si>
-  <si>
-    <t>Alteração no Otimizador 2 considerando os projetos Plano B</t>
-  </si>
-  <si>
-    <t>Visibilidade e Acompanhamento de indicadores relacionados à prodidão</t>
-  </si>
-  <si>
-    <t>Mensurar o impacto da implementação da prorrogação</t>
-  </si>
-  <si>
-    <t>Criar 4 relatórios com dados para suportar decisões de prontidão</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gestão de Processo </t>
-  </si>
-  <si>
-    <t>Olhar o longo prazo avaliando otimizador 2</t>
-  </si>
-  <si>
-    <t>[OTM2] Feature mais de uma regra de inicio de projeto por municipio</t>
-  </si>
-  <si>
-    <t>[GATE 2] Calcular prontidão por contratada e região (Novo Filtro)</t>
-  </si>
-  <si>
-    <t>[Melhoria][Média] Criar uma lista de exceções para o Otimizador 2</t>
-  </si>
-  <si>
-    <t>[Melhoria][Media] Identificar automaticamente gargalos por semana, região ou fase</t>
-  </si>
-  <si>
-    <t>[Melhoria][Baixo] Introduzir bandas de custo na função objetivo</t>
-  </si>
-  <si>
-    <t>Should Cost</t>
-  </si>
-  <si>
-    <t>Visibilidade de indicadores Shoud Cost</t>
-  </si>
-  <si>
-    <t>Automatizar indicadores no output dos planos gerados nas rodadas de otimização</t>
-  </si>
-  <si>
-    <t>Exibição de indicadores executivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criar ferramenta visual de comparação de should cost entre os planos </t>
-  </si>
-  <si>
-    <t>Expansão de escopo</t>
-  </si>
-  <si>
-    <t>[Melhoria][Baixo +] Adicionar escopo de vala aberta / loteamento</t>
-  </si>
-  <si>
-    <t>Simulador de Should Cost</t>
-  </si>
-  <si>
-    <t>Funcionalidade para simulações de cenários de Should Cost</t>
-  </si>
-  <si>
-    <t>Criar output executivo replicando premissas da calculadora do Negocia+ (Suprimentos)</t>
+    <t>Arquivos no Sharepoint</t>
   </si>
   <si>
     <t>Capacity</t>
@@ -638,7 +669,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -707,9 +738,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -808,6 +836,7 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Rafael Amancio Diegues" id="{91DE2057-FAF3-44A7-B512-91FAE0BD3E56}" userId="S::TR069373@comgas.com.br::097fe6cb-a905-47b4-835c-5c8e36db22b1" providerId="AD"/>
+  <person displayName="Marcelo Langhinrichs Cunha" id="{469A5450-6BD5-4D95-88E0-A17096FDFA3B}" userId="S::tr062660@comgas.com.br::c26e65b1-ba35-454a-9a05-e190cb094112" providerId="AD"/>
 </personList>
 </file>
 
@@ -1128,6 +1157,20 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C5" dT="2026-03-18T12:13:24.51" personId="{469A5450-6BD5-4D95-88E0-A17096FDFA3B}" id="{5E7ADAE3-BFAF-4354-AE7C-4DA203F90938}" done="1">
+    <text>Eu subiria um pouco de prioridade (talvez 2) os épicos de sistematização porque eles podem ajudar na conformidade e no tempo de gerar as MFs. No frontend alguns filtros básicos já podem ser feitos para garantir menos problemas de ingestão ou dados errados.
+De todo modo esses desenvolvimentos tem um pouco menos de competição pelo tipo de recurso que utiliza, e devem ser feitos no futuro mais próximo</text>
+  </threadedComment>
+  <threadedComment ref="C5" dT="2026-03-18T13:32:15.61" personId="{91DE2057-FAF3-44A7-B512-91FAE0BD3E56}" id="{02F27FFC-0A39-4455-91A5-8B7C6FFA140A}" parentId="{5E7ADAE3-BFAF-4354-AE7C-4DA203F90938}">
+    <text>Concordo. Subi aqui a prioridade. Temos que avaliar porque temos uma sequência grande de homologações travadas já, mas acho que vale o push para o time de negócio.</text>
+  </threadedComment>
+  <threadedComment ref="C13" dT="2026-03-18T12:07:08.34" personId="{469A5450-6BD5-4D95-88E0-A17096FDFA3B}" id="{C17263A4-E425-444C-BF97-70B1448F129A}" done="1">
+    <text>Acredito que esse item por estar quente e afetar algumas respostas na visão de prontidão, podem ser mais prioritário no OTM2 que aquela questão de bandas na na função objetivo que ficou com prioridade 1. Eu as inverteria</text>
+  </threadedComment>
+  <threadedComment ref="C32" dT="2026-03-18T12:11:19.79" personId="{469A5450-6BD5-4D95-88E0-A17096FDFA3B}" id="{4ACDD4B6-EB3F-4684-99D5-3EA6906C96CE}">
+    <text>Eu entendi o ponto das features de monitoramente estejam a frente das de produtização que são 100% técnicas, porque elas trazem valor pro time de negócio.
+Eu só levaria em conta o risco de demorar a produtização técnica e isso poder ficar muito pra frente e ter problemas de orçamento ano que vem. Mas do ponto de vista de negócios, estou de acordo com a ordem</text>
+  </threadedComment>
   <threadedComment ref="C53" dT="2026-03-17T15:01:51.58" personId="{91DE2057-FAF3-44A7-B512-91FAE0BD3E56}" id="{5050488C-96D1-43A8-9998-3148830ABB2C}">
     <text>A princípio, não será realizado, dada sistematização e integração</text>
   </threadedComment>
@@ -1136,7 +1179,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1149,7 +1191,7 @@
     <col min="8" max="8" width="22.85546875" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="15.140625" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" style="36" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="35" customWidth="1"/>
     <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1184,22 +1226,22 @@
       <c r="J1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="35" t="s">
+      <c r="K1" s="34" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>15</v>
@@ -1223,20 +1265,20 @@
       <c r="J2" s="17">
         <v>1</v>
       </c>
-      <c r="K2" s="36">
+      <c r="K2" s="35">
         <f t="shared" ref="K2:K33" si="1">(6-J2)^1.5/((I2+0.01)^0.5)*100</f>
         <v>298.70049262920656</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>15</v>
@@ -1260,20 +1302,20 @@
       <c r="J3" s="17">
         <v>1</v>
       </c>
-      <c r="K3" s="36">
+      <c r="K3" s="35">
         <f t="shared" si="1"/>
         <v>186.31312309908182</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>15</v>
@@ -1297,366 +1339,366 @@
       <c r="J4" s="17">
         <v>1</v>
       </c>
-      <c r="K4" s="36">
+      <c r="K4" s="35">
         <f t="shared" si="1"/>
         <v>181.34520288620678</v>
       </c>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E5" s="2">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="F5" s="3">
         <v>0</v>
       </c>
       <c r="G5" s="3">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H5" s="3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I5" s="17">
         <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="J5" s="17">
+        <v>2</v>
+      </c>
+      <c r="K5" s="35">
+        <f t="shared" si="1"/>
+        <v>178.84073360395831</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="2">
+        <v>6</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <v>12</v>
+      </c>
+      <c r="H6" s="3">
+        <v>2</v>
+      </c>
+      <c r="I6" s="17">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="J6" s="17">
+        <v>2</v>
+      </c>
+      <c r="K6" s="35">
+        <f t="shared" si="1"/>
+        <v>178.84073360395831</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2">
+        <v>6</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>12</v>
+      </c>
+      <c r="H7" s="3">
+        <v>2</v>
+      </c>
+      <c r="I7" s="17">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="J7" s="17">
+        <v>2</v>
+      </c>
+      <c r="K7" s="35">
+        <f t="shared" si="1"/>
+        <v>178.84073360395831</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2">
+        <v>6</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>12</v>
+      </c>
+      <c r="H8" s="3">
+        <v>2</v>
+      </c>
+      <c r="I8" s="17">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="J8" s="17">
+        <v>2</v>
+      </c>
+      <c r="K8" s="35">
+        <f t="shared" si="1"/>
+        <v>178.84073360395831</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2">
+        <v>30</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>12</v>
+      </c>
+      <c r="I9" s="17">
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J9" s="17">
         <v>1</v>
       </c>
-      <c r="K5" s="36">
+      <c r="K9" s="35">
         <f t="shared" si="1"/>
         <v>172.49585583684464</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="2">
-        <v>12</v>
-      </c>
-      <c r="F6" s="3">
-        <v>12</v>
-      </c>
-      <c r="G6" s="3">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3">
-        <v>2</v>
-      </c>
-      <c r="I6" s="17">
-        <f t="shared" si="0"/>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J6" s="17">
-        <v>2</v>
-      </c>
-      <c r="K6" s="36">
-        <f t="shared" si="1"/>
-        <v>156.86274509803917</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="C10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E10" s="2">
         <v>30</v>
       </c>
-      <c r="F7" s="3">
-        <v>0</v>
-      </c>
-      <c r="G7" s="3">
-        <v>12</v>
-      </c>
-      <c r="H7" s="3">
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
+        <v>12</v>
+      </c>
+      <c r="H10" s="3">
         <v>18</v>
       </c>
-      <c r="I7" s="17">
+      <c r="I10" s="17">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="J7" s="17">
+      <c r="J10" s="17">
         <v>1</v>
       </c>
-      <c r="K7" s="36">
+      <c r="K10" s="35">
         <f t="shared" si="1"/>
         <v>144.32554067010582</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="2">
+    <row r="11" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="2">
         <v>6</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F11" s="3">
         <v>24</v>
       </c>
-      <c r="G8" s="3">
-        <v>0</v>
-      </c>
-      <c r="H8" s="3">
+      <c r="G11" s="3">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3">
         <v>2</v>
       </c>
-      <c r="I8" s="17">
+      <c r="I11" s="17">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="J8" s="17">
+      <c r="J11" s="17">
         <v>2</v>
       </c>
-      <c r="K8" s="36">
+      <c r="K11" s="35">
         <f t="shared" si="1"/>
         <v>141.39926432805382</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="45" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="2">
-        <v>12</v>
-      </c>
-      <c r="F9" s="3">
+    <row r="12" spans="1:12" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="2">
+        <v>12</v>
+      </c>
+      <c r="F12" s="3">
         <f>8*6</f>
         <v>48</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G12" s="3">
         <v>6</v>
       </c>
-      <c r="H9" s="3">
-        <v>12</v>
-      </c>
-      <c r="I9" s="17">
+      <c r="H12" s="3">
+        <v>12</v>
+      </c>
+      <c r="I12" s="17">
         <f t="shared" si="0"/>
         <v>78</v>
       </c>
-      <c r="J9" s="17">
+      <c r="J12" s="17">
         <v>1</v>
       </c>
-      <c r="K9" s="36">
+      <c r="K12" s="35">
         <f t="shared" si="1"/>
         <v>126.58430676687897</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3">
-        <v>18</v>
-      </c>
-      <c r="G10" s="3">
-        <v>0</v>
-      </c>
-      <c r="H10" s="3">
-        <v>2</v>
-      </c>
-      <c r="I10" s="17">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="J10" s="17">
-        <v>3</v>
-      </c>
-      <c r="K10" s="36">
-        <f t="shared" si="1"/>
-        <v>116.16046389935495</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="2">
-        <v>6</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3">
-        <v>12</v>
-      </c>
-      <c r="H11" s="3">
-        <v>2</v>
-      </c>
-      <c r="I11" s="17">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="J11" s="17">
-        <v>3</v>
-      </c>
-      <c r="K11" s="36">
-        <f t="shared" si="1"/>
-        <v>116.16046389935495</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="35.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="2">
-        <v>6</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0</v>
-      </c>
-      <c r="G12" s="3">
-        <v>12</v>
-      </c>
-      <c r="H12" s="3">
-        <v>2</v>
-      </c>
-      <c r="I12" s="17">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="J12" s="17">
-        <v>3</v>
-      </c>
-      <c r="K12" s="36">
-        <f t="shared" si="1"/>
-        <v>116.16046389935495</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F13" s="3">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G13" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H13" s="3">
         <v>2</v>
       </c>
       <c r="I13" s="17">
         <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="J13" s="17">
+        <v>2</v>
+      </c>
+      <c r="K13" s="35">
+        <f t="shared" si="1"/>
+        <v>120.59083510563586</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J13" s="17">
-        <v>3</v>
-      </c>
-      <c r="K13" s="36">
-        <f t="shared" si="1"/>
-        <v>116.16046389935495</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F14" s="3">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G14" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H14" s="3">
         <v>2</v>
@@ -1668,20 +1710,20 @@
       <c r="J14" s="17">
         <v>3</v>
       </c>
-      <c r="K14" s="36">
+      <c r="K14" s="35">
         <f t="shared" si="1"/>
         <v>116.16046389935495</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>15</v>
@@ -1705,20 +1747,20 @@
       <c r="J15" s="17">
         <v>2</v>
       </c>
-      <c r="K15" s="36">
+      <c r="K15" s="35">
         <f t="shared" si="1"/>
         <v>115.45802758638619</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>15</v>
@@ -1742,20 +1784,20 @@
       <c r="J16" s="17">
         <v>2</v>
       </c>
-      <c r="K16" s="36">
+      <c r="K16" s="35">
         <f t="shared" si="1"/>
         <v>106.89495299877967</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>15</v>
@@ -1779,32 +1821,32 @@
       <c r="J17" s="17">
         <v>2</v>
       </c>
-      <c r="K17" s="36">
+      <c r="K17" s="35">
         <f t="shared" si="1"/>
         <v>106.89495299877967</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
+    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>15</v>
+      <c r="D18" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="E18" s="2">
         <v>12</v>
       </c>
       <c r="F18" s="3">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G18" s="3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H18" s="3">
         <v>2</v>
@@ -1816,32 +1858,32 @@
       <c r="J18" s="17">
         <v>3</v>
       </c>
-      <c r="K18" s="36">
+      <c r="K18" s="35">
         <f t="shared" si="1"/>
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>63</v>
+    <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>21</v>
+        <v>44</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="E19" s="2">
+        <v>12</v>
+      </c>
+      <c r="F19" s="3">
         <v>6</v>
       </c>
-      <c r="F19" s="3">
-        <v>18</v>
-      </c>
       <c r="G19" s="3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H19" s="3">
         <v>2</v>
@@ -1853,244 +1895,244 @@
       <c r="J19" s="17">
         <v>3</v>
       </c>
-      <c r="K19" s="36">
+      <c r="K19" s="35">
         <f t="shared" si="1"/>
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>65</v>
+        <v>16</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E20" s="2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F20" s="3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G20" s="3">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H20" s="3">
         <v>2</v>
       </c>
       <c r="I20" s="17">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="J20" s="17">
         <v>3</v>
       </c>
-      <c r="K20" s="36">
+      <c r="K20" s="35">
+        <f t="shared" si="1"/>
+        <v>101.88534162169867</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="2">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>12</v>
+      </c>
+      <c r="G21" s="3">
+        <v>18</v>
+      </c>
+      <c r="H21" s="3">
+        <v>2</v>
+      </c>
+      <c r="I21" s="17">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="J21" s="17">
+        <v>3</v>
+      </c>
+      <c r="K21" s="35">
         <f t="shared" si="1"/>
         <v>91.841516238394064</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" s="22" t="s">
+    <row r="22" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E22" s="2">
         <v>24</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F22" s="3">
         <f>4*24</f>
         <v>96</v>
       </c>
-      <c r="G21" s="3">
-        <v>12</v>
-      </c>
-      <c r="H21" s="3">
+      <c r="G22" s="3">
+        <v>12</v>
+      </c>
+      <c r="H22" s="3">
         <f>24</f>
         <v>24</v>
       </c>
-      <c r="I21" s="17">
+      <c r="I22" s="17">
         <f t="shared" si="0"/>
         <v>156</v>
       </c>
-      <c r="J21">
+      <c r="J22">
         <v>1</v>
       </c>
-      <c r="K21" s="36">
+      <c r="K22" s="35">
         <f t="shared" si="1"/>
         <v>89.511490342880691</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D22" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="E22" s="2">
-        <v>12</v>
-      </c>
-      <c r="F22" s="3">
+    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="2">
+        <v>12</v>
+      </c>
+      <c r="F23" s="3">
         <v>24</v>
       </c>
-      <c r="G22" s="3">
-        <v>0</v>
-      </c>
-      <c r="H22" s="3">
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3">
         <v>2</v>
       </c>
-      <c r="I22" s="17">
+      <c r="I23" s="17">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="J22" s="17">
+      <c r="J23" s="17">
         <v>3</v>
       </c>
-      <c r="K22" s="36">
+      <c r="K23" s="35">
         <f t="shared" si="1"/>
         <v>84.281634083146102</v>
       </c>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="2">
         <v>24</v>
       </c>
-      <c r="B23" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="E23" s="2">
-        <v>24</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="3">
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
         <v>6</v>
       </c>
-      <c r="H23" s="3">
-        <v>12</v>
-      </c>
-      <c r="I23" s="17">
+      <c r="H24" s="3">
+        <v>12</v>
+      </c>
+      <c r="I24" s="17">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="J23" s="17">
+      <c r="J24" s="17">
         <v>3</v>
       </c>
-      <c r="K23" s="36">
+      <c r="K24" s="35">
         <f t="shared" si="1"/>
         <v>80.168829233507395</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="1" t="s">
+    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E25" s="2">
         <v>42</v>
       </c>
-      <c r="F24" s="3">
-        <v>12</v>
-      </c>
-      <c r="G24" s="3">
+      <c r="F25" s="3">
+        <v>12</v>
+      </c>
+      <c r="G25" s="3">
         <v>42</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H25" s="3">
         <v>4</v>
       </c>
-      <c r="I24" s="17">
+      <c r="I25" s="17">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="J24" s="17">
+      <c r="J25" s="17">
         <v>2</v>
       </c>
-      <c r="K24" s="36">
+      <c r="K25" s="35">
         <f t="shared" si="1"/>
         <v>79.996000299974995</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E25" s="2">
-        <v>0</v>
-      </c>
-      <c r="F25" s="3">
-        <v>42</v>
-      </c>
-      <c r="G25" s="3">
-        <v>0</v>
-      </c>
-      <c r="H25" s="3">
-        <v>2</v>
-      </c>
-      <c r="I25" s="17">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="J25" s="17">
-        <v>3</v>
-      </c>
-      <c r="K25" s="36">
-        <f t="shared" si="1"/>
-        <v>78.326044998795737</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>15</v>
@@ -2114,23 +2156,23 @@
       <c r="J26" s="17">
         <v>3</v>
       </c>
-      <c r="K26" s="36">
+      <c r="K26" s="35">
         <f t="shared" si="1"/>
         <v>74.992188720491242</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E27" s="2">
         <v>6</v>
@@ -2151,20 +2193,20 @@
       <c r="J27" s="17">
         <v>3</v>
       </c>
-      <c r="K27" s="36">
+      <c r="K27" s="35">
         <f t="shared" si="1"/>
         <v>73.477344916353701</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>15</v>
@@ -2188,20 +2230,20 @@
       <c r="J28" s="17">
         <v>4</v>
       </c>
-      <c r="K28" s="36">
+      <c r="K28" s="35">
         <f t="shared" si="1"/>
         <v>63.229747741867904</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>15</v>
@@ -2225,23 +2267,23 @@
       <c r="J29" s="17">
         <v>4</v>
       </c>
-      <c r="K29" s="36">
+      <c r="K29" s="35">
         <f t="shared" si="1"/>
         <v>55.459355387180189</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="24" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E30" s="2">
         <v>30</v>
@@ -2262,20 +2304,20 @@
       <c r="J30" s="17">
         <v>3</v>
       </c>
-      <c r="K30" s="36">
+      <c r="K30" s="35">
         <f t="shared" si="1"/>
         <v>51.44705369016468</v>
       </c>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>15</v>
@@ -2299,23 +2341,23 @@
       <c r="J31" s="17">
         <v>4</v>
       </c>
-      <c r="K31" s="36">
+      <c r="K31" s="35">
         <f t="shared" si="1"/>
         <v>49.992189330577979</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
@@ -2336,20 +2378,20 @@
       <c r="J32" s="17">
         <v>4</v>
       </c>
-      <c r="K32" s="36">
+      <c r="K32" s="35">
         <f t="shared" si="1"/>
         <v>43.638383310758336</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>15</v>
@@ -2373,23 +2415,23 @@
       <c r="J33" s="17">
         <v>4</v>
       </c>
-      <c r="K33" s="36">
+      <c r="K33" s="35">
         <f t="shared" si="1"/>
         <v>43.638383310758336</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D34" s="34" t="s">
-        <v>21</v>
+      <c r="D34" s="33" t="s">
+        <v>25</v>
       </c>
       <c r="E34" s="2">
         <v>0</v>
@@ -2410,20 +2452,20 @@
       <c r="J34" s="17">
         <v>4</v>
       </c>
-      <c r="K34" s="36">
+      <c r="K34" s="35">
         <f t="shared" ref="K34:K53" si="3">(6-J34)^1.5/((I34+0.01)^0.5)*100</f>
         <v>40.82057712437858</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>15</v>
@@ -2447,20 +2489,20 @@
       <c r="J35" s="17">
         <v>5</v>
       </c>
-      <c r="K35" s="36">
+      <c r="K35" s="35">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>15</v>
@@ -2484,20 +2526,20 @@
       <c r="J36" s="17">
         <v>5</v>
       </c>
-      <c r="K36" s="36">
+      <c r="K36" s="35">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>15</v>
@@ -2521,20 +2563,20 @@
       <c r="J37" s="17">
         <v>5</v>
       </c>
-      <c r="K37" s="36">
+      <c r="K37" s="35">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>15</v>
@@ -2558,20 +2600,20 @@
       <c r="J38" s="17">
         <v>5</v>
       </c>
-      <c r="K38" s="36">
+      <c r="K38" s="35">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>15</v>
@@ -2595,20 +2637,20 @@
       <c r="J39" s="17">
         <v>5</v>
       </c>
-      <c r="K39" s="36">
+      <c r="K39" s="35">
         <f t="shared" si="3"/>
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>15</v>
@@ -2632,20 +2674,20 @@
       <c r="J40" s="17">
         <v>5</v>
       </c>
-      <c r="K40" s="36">
+      <c r="K40" s="35">
         <f t="shared" si="3"/>
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="34.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>15</v>
@@ -2669,23 +2711,23 @@
       <c r="J41" s="17">
         <v>5</v>
       </c>
-      <c r="K41" s="36">
+      <c r="K41" s="35">
         <f t="shared" si="3"/>
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="38.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D42" s="34" t="s">
-        <v>21</v>
+        <v>73</v>
+      </c>
+      <c r="D42" s="33" t="s">
+        <v>25</v>
       </c>
       <c r="E42" s="2">
         <v>0</v>
@@ -2706,20 +2748,20 @@
       <c r="J42" s="17">
         <v>5</v>
       </c>
-      <c r="K42" s="36">
+      <c r="K42" s="35">
         <f t="shared" si="3"/>
         <v>27.724348650071377</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>15</v>
@@ -2743,20 +2785,20 @@
       <c r="J43" s="17">
         <v>5</v>
       </c>
-      <c r="K43" s="36">
+      <c r="K43" s="35">
         <f t="shared" si="3"/>
         <v>26.716584257263243</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>15</v>
@@ -2780,23 +2822,23 @@
       <c r="J44" s="17">
         <v>5</v>
       </c>
-      <c r="K44" s="36">
+      <c r="K44" s="35">
         <f t="shared" si="3"/>
         <v>23.563681481313655</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C45" s="28" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E45" s="27">
         <v>0</v>
@@ -2817,20 +2859,20 @@
       <c r="J45" s="17">
         <v>5</v>
       </c>
-      <c r="K45" s="36">
+      <c r="K45" s="35">
         <f t="shared" si="3"/>
         <v>22.355091700494793</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>15</v>
@@ -2854,20 +2896,20 @@
       <c r="J46" s="17">
         <v>5</v>
       </c>
-      <c r="K46" s="36">
+      <c r="K46" s="35">
         <f t="shared" si="3"/>
         <v>20.408163265306118</v>
       </c>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>15</v>
@@ -2891,23 +2933,23 @@
       <c r="J47" s="17">
         <v>5</v>
       </c>
-      <c r="K47" s="36">
+      <c r="K47" s="35">
         <f t="shared" si="3"/>
         <v>19.6078431372549</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D48" s="34" t="s">
-        <v>21</v>
+        <v>79</v>
+      </c>
+      <c r="D48" s="33" t="s">
+        <v>25</v>
       </c>
       <c r="E48" s="2">
         <v>6</v>
@@ -2928,23 +2970,23 @@
       <c r="J48" s="17">
         <v>5</v>
       </c>
-      <c r="K48" s="36">
+      <c r="K48" s="35">
         <f t="shared" si="3"/>
         <v>18.254376440922808</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D49" s="34" t="s">
-        <v>21</v>
+        <v>80</v>
+      </c>
+      <c r="D49" s="33" t="s">
+        <v>25</v>
       </c>
       <c r="E49" s="2">
         <v>30</v>
@@ -2965,23 +3007,23 @@
       <c r="J49" s="17">
         <v>5</v>
       </c>
-      <c r="K49" s="36">
+      <c r="K49" s="35">
         <f t="shared" si="3"/>
         <v>17.674908041006731</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="D50" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E50" s="27">
         <v>12</v>
@@ -3002,23 +3044,23 @@
       <c r="J50" s="17">
         <v>5</v>
       </c>
-      <c r="K50" s="36">
+      <c r="K50" s="35">
         <f t="shared" si="3"/>
         <v>16.664352333993332</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D51" s="34" t="s">
-        <v>21</v>
+        <v>82</v>
+      </c>
+      <c r="D51" s="33" t="s">
+        <v>25</v>
       </c>
       <c r="E51" s="2">
         <v>12</v>
@@ -3039,20 +3081,20 @@
       <c r="J51" s="17">
         <v>5</v>
       </c>
-      <c r="K51" s="36">
+      <c r="K51" s="35">
         <f t="shared" si="3"/>
         <v>15.073854388204486</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>15</v>
@@ -3076,20 +3118,20 @@
       <c r="J52" s="17">
         <v>5</v>
       </c>
-      <c r="K52" s="36">
+      <c r="K52" s="35">
         <f t="shared" si="3"/>
         <v>8.7035531239860209</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>15</v>
@@ -3113,22 +3155,13 @@
       <c r="J53" s="17">
         <v>5</v>
       </c>
-      <c r="K53" s="36">
+      <c r="K53" s="35">
         <f t="shared" si="3"/>
         <v>4.472091234310839</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L53" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="N/A"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L53">
-      <sortCondition descending="1" ref="K1:K53"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:L53" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Aptos"&amp;10&amp;K000000 Interno&amp;1#_x000D_</oddHeader>
@@ -3319,15 +3352,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010023E2413248AD144EB4F352681303D788" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e915d9c603a07a4fc4694295454b5583">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="898695ca-150f-4d53-a1a4-27c213b72f41" xmlns:ns3="11e3fce6-e222-4248-a00d-b3b33ed830c1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b1e7ba0d6315b4b8ad6fa6ed50b7c17a" ns2:_="" ns3:_="">
     <xsd:import namespace="898695ca-150f-4d53-a1a4-27c213b72f41"/>
@@ -3522,7 +3546,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="898695ca-150f-4d53-a1a4-27c213b72f41">
@@ -3533,15 +3557,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0855675D-7A7E-4EB6-A046-05A9ACCF1C10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{591A5FB6-33BD-4B1F-88D8-436DAE7CA680}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3560,19 +3585,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94EFCDE8-B628-4468-B13F-930C6557CB2F}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="898695ca-150f-4d53-a1a4-27c213b72f41"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="11e3fce6-e222-4248-a00d-b3b33ed830c1"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="898695ca-150f-4d53-a1a4-27c213b72f41"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="11e3fce6-e222-4248-a00d-b3b33ed830c1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0855675D-7A7E-4EB6-A046-05A9ACCF1C10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: Simplify filters and frontend toggle
</commit_message>
<xml_diff>
--- a/Backlog_Roadmap_2026.xlsx
+++ b/Backlog_Roadmap_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Consultor Noorden\Desktop\planning-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858D3C0E-6270-46C7-94DE-212C6DEA8FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4F990E-91EE-4535-B6FF-940F746F4DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="104">
   <si>
     <t>Indicadores</t>
   </si>
@@ -151,9 +151,6 @@
     <t>Should Cost</t>
   </si>
   <si>
-    <t>Visibilidade de indicadores Shoud Cost</t>
-  </si>
-  <si>
     <t>Criar output executivo replicando premissas da calculadora do Negocia+ (Suprimentos)</t>
   </si>
   <si>
@@ -169,9 +166,6 @@
     <t>Backlog Parting Lote-BCG</t>
   </si>
   <si>
-    <t>Visibilidade e Acompanhamento de indicadores relacionados à prodidão</t>
-  </si>
-  <si>
     <t>Mensurar o impacto da implementação da prorrogação</t>
   </si>
   <si>
@@ -242,9 +236,6 @@
   </si>
   <si>
     <t>Aderência</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visibilidade de idicadoes de Aderência </t>
   </si>
   <si>
     <t>Disponibilizar para o time de negócio um dashboard de Aderencia</t>
@@ -409,6 +400,9 @@
   </si>
   <si>
     <t>Resultados em horas</t>
+  </si>
+  <si>
+    <t>Visibilidade de indicadores</t>
   </si>
 </sst>
 </file>
@@ -1179,6 +1173,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1233,7 +1228,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>12</v>
       </c>
@@ -1270,7 +1265,7 @@
         <v>298.70049262920656</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>16</v>
       </c>
@@ -1307,15 +1302,15 @@
         <v>186.31312309908182</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>15</v>
@@ -1344,15 +1339,15 @@
         <v>181.34520288620678</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>15</v>
@@ -1381,15 +1376,15 @@
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>15</v>
@@ -1418,15 +1413,15 @@
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>15</v>
@@ -1455,15 +1450,15 @@
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>15</v>
@@ -1492,7 +1487,7 @@
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>12</v>
       </c>
@@ -1500,7 +1495,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>15</v>
@@ -1529,15 +1524,15 @@
         <v>172.49585583684464</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>26</v>
+        <v>103</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>15</v>
@@ -1566,18 +1561,18 @@
         <v>144.32554067010582</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="D11" s="29" t="s">
         <v>29</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>31</v>
       </c>
       <c r="E11" s="2">
         <v>6</v>
@@ -1603,18 +1598,18 @@
         <v>141.39926432805382</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="35.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="2">
         <v>12</v>
@@ -1641,15 +1636,15 @@
         <v>126.58430676687897</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>15</v>
@@ -1678,15 +1673,15 @@
         <v>120.59083510563586</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>20</v>
+        <v>103</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>15</v>
@@ -1715,15 +1710,15 @@
         <v>116.16046389935495</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>20</v>
+        <v>103</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>15</v>
@@ -1752,15 +1747,15 @@
         <v>115.45802758638619</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>15</v>
@@ -1789,15 +1784,15 @@
         <v>106.89495299877967</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>15</v>
@@ -1826,18 +1821,18 @@
         <v>106.89495299877967</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="15" t="s">
         <v>24</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>25</v>
       </c>
       <c r="E18" s="2">
         <v>12</v>
@@ -1863,15 +1858,15 @@
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>15</v>
@@ -1900,18 +1895,18 @@
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E20" s="2">
         <v>6</v>
@@ -1937,18 +1932,18 @@
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="14" t="s">
-        <v>26</v>
+      <c r="B21" s="1" t="s">
+        <v>103</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E21" s="2">
         <v>0</v>
@@ -1974,15 +1969,15 @@
         <v>91.841516238394064</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="14" t="s">
-        <v>26</v>
+      <c r="B22" s="1" t="s">
+        <v>103</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>15</v>
@@ -2013,18 +2008,18 @@
         <v>89.511490342880691</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
         <v>16</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E23" s="2">
         <v>12</v>
@@ -2050,15 +2045,15 @@
         <v>84.281634083146102</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>15</v>
@@ -2087,15 +2082,15 @@
         <v>80.168829233507395</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>51</v>
+        <v>103</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>15</v>
@@ -2124,15 +2119,15 @@
         <v>79.996000299974995</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>19</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>15</v>
@@ -2161,18 +2156,18 @@
         <v>74.992188720491242</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27" s="2">
         <v>6</v>
@@ -2198,15 +2193,15 @@
         <v>73.477344916353701</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>20</v>
+        <v>103</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>15</v>
@@ -2235,15 +2230,15 @@
         <v>63.229747741867904</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>15</v>
@@ -2272,18 +2267,18 @@
         <v>55.459355387180189</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E30" s="2">
         <v>30</v>
@@ -2309,15 +2304,15 @@
         <v>51.44705369016468</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>15</v>
@@ -2346,18 +2341,18 @@
         <v>49.992189330577979</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
         <v>12</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
@@ -2383,15 +2378,15 @@
         <v>43.638383310758336</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>15</v>
@@ -2420,18 +2415,18 @@
         <v>43.638383310758336</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>16</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>26</v>
+        <v>103</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D34" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E34" s="2">
         <v>0</v>
@@ -2457,15 +2452,15 @@
         <v>40.82057712437858</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D35" s="30" t="s">
         <v>15</v>
@@ -2494,15 +2489,15 @@
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>15</v>
@@ -2531,15 +2526,15 @@
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>15</v>
@@ -2568,15 +2563,15 @@
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>15</v>
@@ -2605,15 +2600,15 @@
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D39" s="30" t="s">
         <v>15</v>
@@ -2642,15 +2637,15 @@
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>15</v>
@@ -2679,15 +2674,15 @@
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="34.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D41" s="30" t="s">
         <v>15</v>
@@ -2716,18 +2711,18 @@
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="38.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
         <v>12</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D42" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E42" s="2">
         <v>0</v>
@@ -2753,15 +2748,15 @@
         <v>27.724348650071377</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>15</v>
@@ -2790,15 +2785,15 @@
         <v>26.716584257263243</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>15</v>
@@ -2827,18 +2822,18 @@
         <v>23.563681481313655</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
         <v>12</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C45" s="28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D45" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E45" s="27">
         <v>0</v>
@@ -2864,15 +2859,15 @@
         <v>22.355091700494793</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>15</v>
@@ -2901,7 +2896,7 @@
         <v>20.408163265306118</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>12</v>
       </c>
@@ -2909,7 +2904,7 @@
         <v>13</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>15</v>
@@ -2938,18 +2933,18 @@
         <v>19.6078431372549</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
         <v>12</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D48" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E48" s="2">
         <v>6</v>
@@ -2975,18 +2970,18 @@
         <v>18.254376440922808</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
         <v>12</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E49" s="2">
         <v>30</v>
@@ -3012,18 +3007,18 @@
         <v>17.674908041006731</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D50" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E50" s="27">
         <v>12</v>
@@ -3049,18 +3044,18 @@
         <v>16.664352333993332</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
         <v>12</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D51" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E51" s="2">
         <v>12</v>
@@ -3086,15 +3081,15 @@
         <v>15.073854388204486</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D52" s="30" t="s">
         <v>15</v>
@@ -3123,15 +3118,15 @@
         <v>8.7035531239860209</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>15</v>
@@ -3161,7 +3156,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L53" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}"/>
+  <autoFilter ref="A1:L53" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="N/A"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Aptos"&amp;10&amp;K000000 Interno&amp;1#_x000D_</oddHeader>
@@ -3187,15 +3188,15 @@
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -3203,7 +3204,7 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D6">
         <v>6</v>
@@ -3211,7 +3212,7 @@
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -3219,7 +3220,7 @@
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -3227,7 +3228,7 @@
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -3235,7 +3236,7 @@
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D10">
         <v>6</v>
@@ -3243,7 +3244,7 @@
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D11" s="5">
         <f>SUM(D5:D10)</f>
@@ -3252,25 +3253,25 @@
     </row>
     <row r="12" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C12">
         <v>10</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E12" s="6">
         <f>(D11*C12-C21)</f>
         <v>268</v>
       </c>
       <c r="I12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D13" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E13" s="6">
         <f>(E12*2)</f>
@@ -3279,7 +3280,7 @@
     </row>
     <row r="14" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D14" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E14" s="6">
         <f>(E13*3)</f>
@@ -3288,13 +3289,13 @@
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C17" s="10">
         <v>1</v>
@@ -3302,7 +3303,7 @@
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C18" s="10">
         <v>6</v>
@@ -3310,7 +3311,7 @@
     </row>
     <row r="19" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C19" s="10">
         <v>4</v>
@@ -3318,7 +3319,7 @@
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C20" s="10">
         <v>1</v>
@@ -3333,12 +3334,12 @@
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -3547,6 +3548,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="898695ca-150f-4d53-a1a4-27c213b72f41">
@@ -3555,15 +3565,6 @@
     <TaxCatchAll xmlns="11e3fce6-e222-4248-a00d-b3b33ed830c1" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3586,26 +3587,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94EFCDE8-B628-4468-B13F-930C6557CB2F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0855675D-7A7E-4EB6-A046-05A9ACCF1C10}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="898695ca-150f-4d53-a1a4-27c213b72f41"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="11e3fce6-e222-4248-a00d-b3b33ed830c1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0855675D-7A7E-4EB6-A046-05A9ACCF1C10}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94EFCDE8-B628-4468-B13F-930C6557CB2F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="11e3fce6-e222-4248-a00d-b3b33ed830c1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="898695ca-150f-4d53-a1a4-27c213b72f41"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: Filter invalid epics
</commit_message>
<xml_diff>
--- a/Backlog_Roadmap_2026.xlsx
+++ b/Backlog_Roadmap_2026.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Consultor Noorden\Desktop\planning-tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Consultor Noorden\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4F990E-91EE-4535-B6FF-940F746F4DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B97E29A-4869-41E7-9D01-7F0E303EDE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="2" r:id="rId1"/>
-    <sheet name="Capacity_Velocity(horas)" sheetId="1" r:id="rId2"/>
+    <sheet name="Capacity_Velocity(horas)" sheetId="1" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$L$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$L$61</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="113">
   <si>
     <t>Indicadores</t>
   </si>
@@ -191,9 +191,6 @@
   </si>
   <si>
     <t>Sistematização</t>
-  </si>
-  <si>
-    <t>Sistematização dos dados de RDO(Relatório diarios de obras)</t>
   </si>
   <si>
     <t>Sistematização das informações de assentamentos</t>
@@ -339,6 +336,33 @@
     <t>Arquivos no Sharepoint</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>[Melhoria][Média] Criar função objetivo por região</t>
+  </si>
+  <si>
+    <t>Incluir financeiros dos projetos e sinalizar estornos de CAPEX, indicando necessidade de reaprovação</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixo] Implementar restrições regionais de capacidade</t>
+  </si>
+  <si>
+    <t>[Melhoria][Medio] Adicionar chance de atraso baseada em histórico e trazer para função objetivo</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixa] Adicionar custo de mudança em relação a execuções anteriores</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixa] Modelar durações mínimas e máximas flexíveis por fase, com penalização por esticar/encurtar</t>
+  </si>
+  <si>
+    <t>[Melhoria][Baixo] Quebrar a decisão final em fases intermediárias (permitir decisão por fase)</t>
+  </si>
+  <si>
+    <t>[Melhoria][Medio] Gerar relatório pós-leitura automaticamente</t>
+  </si>
+  <si>
     <t>Capacity</t>
   </si>
   <si>
@@ -403,6 +427,9 @@
   </si>
   <si>
     <t>Visibilidade de indicadores</t>
+  </si>
+  <si>
+    <t>Sistematização dos dados de RDO</t>
   </si>
 </sst>
 </file>
@@ -498,7 +525,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -659,11 +686,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -729,6 +767,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1173,8 +1220,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="34.42578125" customWidth="1"/>
@@ -1186,7 +1232,7 @@
     <col min="8" max="8" width="22.85546875" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="15.140625" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" style="35" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="38" customWidth="1"/>
     <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1221,14 +1267,14 @@
       <c r="J1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="34" t="s">
+      <c r="K1" s="37" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>12</v>
       </c>
@@ -1260,12 +1306,12 @@
       <c r="J2" s="17">
         <v>1</v>
       </c>
-      <c r="K2" s="35">
+      <c r="K2" s="38">
         <f t="shared" ref="K2:K33" si="1">(6-J2)^1.5/((I2+0.01)^0.5)*100</f>
         <v>298.70049262920656</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>16</v>
       </c>
@@ -1297,17 +1343,17 @@
       <c r="J3" s="17">
         <v>1</v>
       </c>
-      <c r="K3" s="35">
+      <c r="K3" s="38">
         <f t="shared" si="1"/>
         <v>186.31312309908182</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>20</v>
@@ -1334,12 +1380,12 @@
       <c r="J4" s="17">
         <v>1</v>
       </c>
-      <c r="K4" s="35">
+      <c r="K4" s="38">
         <f t="shared" si="1"/>
         <v>181.34520288620678</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>12</v>
       </c>
@@ -1347,7 +1393,7 @@
         <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>34</v>
+        <v>112</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>15</v>
@@ -1371,12 +1417,12 @@
       <c r="J5" s="17">
         <v>2</v>
       </c>
-      <c r="K5" s="35">
+      <c r="K5" s="38">
         <f t="shared" si="1"/>
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>12</v>
       </c>
@@ -1384,7 +1430,7 @@
         <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>15</v>
@@ -1408,12 +1454,12 @@
       <c r="J6" s="17">
         <v>2</v>
       </c>
-      <c r="K6" s="35">
+      <c r="K6" s="38">
         <f t="shared" si="1"/>
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>12</v>
       </c>
@@ -1421,7 +1467,7 @@
         <v>33</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>15</v>
@@ -1445,12 +1491,12 @@
       <c r="J7" s="17">
         <v>2</v>
       </c>
-      <c r="K7" s="35">
+      <c r="K7" s="38">
         <f t="shared" si="1"/>
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>12</v>
       </c>
@@ -1458,7 +1504,7 @@
         <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>15</v>
@@ -1482,12 +1528,12 @@
       <c r="J8" s="17">
         <v>2</v>
       </c>
-      <c r="K8" s="35">
+      <c r="K8" s="38">
         <f t="shared" si="1"/>
         <v>178.84073360395831</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>12</v>
       </c>
@@ -1519,17 +1565,17 @@
       <c r="J9" s="17">
         <v>1</v>
       </c>
-      <c r="K9" s="35">
+      <c r="K9" s="38">
         <f t="shared" si="1"/>
         <v>172.49585583684464</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>25</v>
@@ -1556,12 +1602,12 @@
       <c r="J10" s="17">
         <v>1</v>
       </c>
-      <c r="K10" s="35">
+      <c r="K10" s="38">
         <f t="shared" si="1"/>
         <v>144.32554067010582</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
         <v>26</v>
       </c>
@@ -1593,12 +1639,12 @@
       <c r="J11" s="17">
         <v>2</v>
       </c>
-      <c r="K11" s="35">
+      <c r="K11" s="38">
         <f t="shared" si="1"/>
         <v>141.39926432805382</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="35.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
         <v>12</v>
       </c>
@@ -1631,12 +1677,12 @@
       <c r="J12" s="17">
         <v>1</v>
       </c>
-      <c r="K12" s="35">
+      <c r="K12" s="38">
         <f t="shared" si="1"/>
         <v>126.58430676687897</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>16</v>
       </c>
@@ -1644,7 +1690,7 @@
         <v>22</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>15</v>
@@ -1668,17 +1714,17 @@
       <c r="J13" s="17">
         <v>2</v>
       </c>
-      <c r="K13" s="35">
+      <c r="K13" s="38">
         <f t="shared" si="1"/>
         <v>120.59083510563586</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>32</v>
@@ -1705,20 +1751,20 @@
       <c r="J14" s="17">
         <v>3</v>
       </c>
-      <c r="K14" s="35">
+      <c r="K14" s="38">
         <f t="shared" si="1"/>
         <v>116.16046389935495</v>
       </c>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>15</v>
@@ -1742,12 +1788,12 @@
       <c r="J15" s="17">
         <v>2</v>
       </c>
-      <c r="K15" s="35">
+      <c r="K15" s="38">
         <f t="shared" si="1"/>
         <v>115.45802758638619</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>26</v>
       </c>
@@ -1755,7 +1801,7 @@
         <v>27</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>15</v>
@@ -1779,12 +1825,12 @@
       <c r="J16" s="17">
         <v>2</v>
       </c>
-      <c r="K16" s="35">
+      <c r="K16" s="38">
         <f t="shared" si="1"/>
         <v>106.89495299877967</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>26</v>
       </c>
@@ -1792,7 +1838,7 @@
         <v>27</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>15</v>
@@ -1816,12 +1862,12 @@
       <c r="J17" s="17">
         <v>2</v>
       </c>
-      <c r="K17" s="35">
+      <c r="K17" s="38">
         <f t="shared" si="1"/>
         <v>106.89495299877967</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>16</v>
       </c>
@@ -1853,20 +1899,20 @@
       <c r="J18" s="17">
         <v>3</v>
       </c>
-      <c r="K18" s="35">
+      <c r="K18" s="38">
         <f t="shared" si="1"/>
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>15</v>
@@ -1890,12 +1936,12 @@
       <c r="J19" s="17">
         <v>3</v>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="38">
         <f t="shared" si="1"/>
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
         <v>16</v>
       </c>
@@ -1903,7 +1949,7 @@
         <v>22</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>24</v>
@@ -1927,22 +1973,22 @@
       <c r="J20" s="17">
         <v>3</v>
       </c>
-      <c r="K20" s="35">
+      <c r="K20" s="38">
         <f t="shared" si="1"/>
         <v>101.88534162169867</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>16</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="35" t="s">
         <v>24</v>
       </c>
       <c r="E21" s="2">
@@ -1964,20 +2010,20 @@
       <c r="J21" s="17">
         <v>3</v>
       </c>
-      <c r="K21" s="35">
+      <c r="K21" s="38">
         <f t="shared" si="1"/>
         <v>91.841516238394064</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>16</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>15</v>
@@ -2003,12 +2049,12 @@
       <c r="J22">
         <v>1</v>
       </c>
-      <c r="K22" s="35">
+      <c r="K22" s="38">
         <f t="shared" si="1"/>
         <v>89.511490342880691</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
         <v>16</v>
       </c>
@@ -2016,9 +2062,9 @@
         <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D23" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="35" t="s">
         <v>24</v>
       </c>
       <c r="E23" s="2">
@@ -2040,20 +2086,20 @@
       <c r="J23" s="17">
         <v>3</v>
       </c>
-      <c r="K23" s="35">
+      <c r="K23" s="38">
         <f t="shared" si="1"/>
         <v>84.281634083146102</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="31" t="s">
-        <v>47</v>
+        <v>40</v>
+      </c>
+      <c r="C24" s="34" t="s">
+        <v>46</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>15</v>
@@ -2077,20 +2123,20 @@
       <c r="J24" s="17">
         <v>3</v>
       </c>
-      <c r="K24" s="35">
+      <c r="K24" s="38">
         <f t="shared" si="1"/>
         <v>80.168829233507395</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>15</v>
@@ -2114,20 +2160,20 @@
       <c r="J25" s="17">
         <v>2</v>
       </c>
-      <c r="K25" s="35">
+      <c r="K25" s="38">
         <f t="shared" si="1"/>
         <v>79.996000299974995</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>19</v>
       </c>
       <c r="B26" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>15</v>
@@ -2151,12 +2197,12 @@
       <c r="J26" s="17">
         <v>3</v>
       </c>
-      <c r="K26" s="35">
+      <c r="K26" s="38">
         <f t="shared" si="1"/>
         <v>74.992188720491242</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>26</v>
       </c>
@@ -2164,7 +2210,7 @@
         <v>27</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>24</v>
@@ -2188,20 +2234,20 @@
       <c r="J27" s="17">
         <v>3</v>
       </c>
-      <c r="K27" s="35">
+      <c r="K27" s="38">
         <f t="shared" si="1"/>
         <v>73.477344916353701</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="36.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C28" s="30" t="s">
-        <v>54</v>
+        <v>111</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>53</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>15</v>
@@ -2225,20 +2271,20 @@
       <c r="J28" s="17">
         <v>4</v>
       </c>
-      <c r="K28" s="35">
+      <c r="K28" s="38">
         <f t="shared" si="1"/>
         <v>63.229747741867904</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>15</v>
@@ -2262,20 +2308,20 @@
       <c r="J29" s="17">
         <v>4</v>
       </c>
-      <c r="K29" s="35">
+      <c r="K29" s="38">
         <f t="shared" si="1"/>
         <v>55.459355387180189</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B30" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>24</v>
@@ -2299,20 +2345,20 @@
       <c r="J30" s="17">
         <v>3</v>
       </c>
-      <c r="K30" s="35">
+      <c r="K30" s="38">
         <f t="shared" si="1"/>
         <v>51.44705369016468</v>
       </c>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>15</v>
@@ -2336,20 +2382,20 @@
       <c r="J31" s="17">
         <v>4</v>
       </c>
-      <c r="K31" s="35">
+      <c r="K31" s="38">
         <f t="shared" si="1"/>
         <v>49.992189330577979</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="32.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
         <v>12</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>24</v>
@@ -2373,20 +2419,20 @@
       <c r="J32" s="17">
         <v>4</v>
       </c>
-      <c r="K32" s="35">
+      <c r="K32" s="38">
         <f t="shared" si="1"/>
         <v>43.638383310758336</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>15</v>
@@ -2410,22 +2456,22 @@
       <c r="J33" s="17">
         <v>4</v>
       </c>
-      <c r="K33" s="35">
+      <c r="K33" s="38">
         <f t="shared" si="1"/>
         <v>43.638383310758336</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>16</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D34" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="36" t="s">
         <v>24</v>
       </c>
       <c r="E34" s="2">
@@ -2441,18 +2487,18 @@
         <v>12</v>
       </c>
       <c r="I34" s="17">
-        <f t="shared" ref="I34:I53" si="2">SUM(E34:H34)</f>
+        <f t="shared" ref="I34:I61" si="2">SUM(E34:H34)</f>
         <v>48</v>
       </c>
       <c r="J34" s="17">
         <v>4</v>
       </c>
-      <c r="K34" s="35">
-        <f t="shared" ref="K34:K53" si="3">(6-J34)^1.5/((I34+0.01)^0.5)*100</f>
+      <c r="K34" s="38">
+        <f t="shared" ref="K34:K61" si="3">(6-J34)^1.5/((I34+0.01)^0.5)*100</f>
         <v>40.82057712437858</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>12</v>
       </c>
@@ -2460,9 +2506,9 @@
         <v>30</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D35" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E35" s="2">
@@ -2484,12 +2530,12 @@
       <c r="J35" s="17">
         <v>5</v>
       </c>
-      <c r="K35" s="35">
+      <c r="K35" s="38">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>12</v>
       </c>
@@ -2497,9 +2543,9 @@
         <v>30</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D36" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E36" s="2">
@@ -2521,12 +2567,12 @@
       <c r="J36" s="17">
         <v>5</v>
       </c>
-      <c r="K36" s="35">
+      <c r="K36" s="38">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>12</v>
       </c>
@@ -2534,9 +2580,9 @@
         <v>30</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D37" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="D37" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E37" s="2">
@@ -2558,12 +2604,12 @@
       <c r="J37" s="17">
         <v>5</v>
       </c>
-      <c r="K37" s="35">
+      <c r="K37" s="38">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>12</v>
       </c>
@@ -2571,9 +2617,9 @@
         <v>30</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D38" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E38" s="2">
@@ -2595,12 +2641,12 @@
       <c r="J38" s="17">
         <v>5</v>
       </c>
-      <c r="K38" s="35">
+      <c r="K38" s="38">
         <f t="shared" si="3"/>
         <v>40.790850822400216</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>12</v>
       </c>
@@ -2608,9 +2654,9 @@
         <v>30</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D39" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E39" s="2">
@@ -2632,12 +2678,12 @@
       <c r="J39" s="17">
         <v>5</v>
       </c>
-      <c r="K39" s="35">
+      <c r="K39" s="38">
         <f t="shared" si="3"/>
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -2645,9 +2691,9 @@
         <v>30</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="D40" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="D40" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E40" s="2">
@@ -2669,12 +2715,12 @@
       <c r="J40" s="17">
         <v>5</v>
       </c>
-      <c r="K40" s="35">
+      <c r="K40" s="38">
         <f t="shared" si="3"/>
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="34.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>12</v>
       </c>
@@ -2682,9 +2728,9 @@
         <v>30</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D41" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="D41" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E41" s="2">
@@ -2706,12 +2752,12 @@
       <c r="J41" s="17">
         <v>5</v>
       </c>
-      <c r="K41" s="35">
+      <c r="K41" s="38">
         <f t="shared" si="3"/>
         <v>28.85549284123806</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="38.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
         <v>12</v>
       </c>
@@ -2719,9 +2765,9 @@
         <v>30</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D42" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="D42" s="36" t="s">
         <v>24</v>
       </c>
       <c r="E42" s="2">
@@ -2743,12 +2789,12 @@
       <c r="J42" s="17">
         <v>5</v>
       </c>
-      <c r="K42" s="35">
+      <c r="K42" s="38">
         <f t="shared" si="3"/>
         <v>27.724348650071377</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>12</v>
       </c>
@@ -2756,9 +2802,9 @@
         <v>30</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D43" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="D43" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E43" s="2">
@@ -2780,12 +2826,12 @@
       <c r="J43" s="17">
         <v>5</v>
       </c>
-      <c r="K43" s="35">
+      <c r="K43" s="38">
         <f t="shared" si="3"/>
         <v>26.716584257263243</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
@@ -2793,9 +2839,9 @@
         <v>30</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D44" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="D44" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E44" s="2">
@@ -2817,12 +2863,12 @@
       <c r="J44" s="17">
         <v>5</v>
       </c>
-      <c r="K44" s="35">
+      <c r="K44" s="38">
         <f t="shared" si="3"/>
         <v>23.563681481313655</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
         <v>12</v>
       </c>
@@ -2830,7 +2876,7 @@
         <v>30</v>
       </c>
       <c r="C45" s="28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D45" t="s">
         <v>29</v>
@@ -2854,12 +2900,12 @@
       <c r="J45" s="17">
         <v>5</v>
       </c>
-      <c r="K45" s="35">
+      <c r="K45" s="38">
         <f t="shared" si="3"/>
         <v>22.355091700494793</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>12</v>
       </c>
@@ -2867,9 +2913,9 @@
         <v>30</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="D46" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="D46" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E46" s="2">
@@ -2891,12 +2937,12 @@
       <c r="J46" s="17">
         <v>5</v>
       </c>
-      <c r="K46" s="35">
+      <c r="K46" s="38">
         <f t="shared" si="3"/>
         <v>20.408163265306118</v>
       </c>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>12</v>
       </c>
@@ -2904,9 +2950,9 @@
         <v>13</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D47" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D47" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E47" s="2">
@@ -2928,12 +2974,12 @@
       <c r="J47" s="17">
         <v>5</v>
       </c>
-      <c r="K47" s="35">
+      <c r="K47" s="38">
         <f t="shared" si="3"/>
         <v>19.6078431372549</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
         <v>12</v>
       </c>
@@ -2941,9 +2987,9 @@
         <v>30</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D48" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48" s="36" t="s">
         <v>24</v>
       </c>
       <c r="E48" s="2">
@@ -2965,12 +3011,12 @@
       <c r="J48" s="17">
         <v>5</v>
       </c>
-      <c r="K48" s="35">
+      <c r="K48" s="38">
         <f t="shared" si="3"/>
         <v>18.254376440922808</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
         <v>12</v>
       </c>
@@ -2978,9 +3024,9 @@
         <v>30</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D49" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="D49" s="36" t="s">
         <v>24</v>
       </c>
       <c r="E49" s="2">
@@ -3002,12 +3048,12 @@
       <c r="J49" s="17">
         <v>5</v>
       </c>
-      <c r="K49" s="35">
+      <c r="K49" s="38">
         <f t="shared" si="3"/>
         <v>17.674908041006731</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>12</v>
       </c>
@@ -3015,7 +3061,7 @@
         <v>30</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D50" t="s">
         <v>29</v>
@@ -3039,12 +3085,12 @@
       <c r="J50" s="17">
         <v>5</v>
       </c>
-      <c r="K50" s="35">
+      <c r="K50" s="38">
         <f t="shared" si="3"/>
         <v>16.664352333993332</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
         <v>12</v>
       </c>
@@ -3052,9 +3098,9 @@
         <v>30</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D51" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="D51" s="36" t="s">
         <v>24</v>
       </c>
       <c r="E51" s="2">
@@ -3076,12 +3122,12 @@
       <c r="J51" s="17">
         <v>5</v>
       </c>
-      <c r="K51" s="35">
+      <c r="K51" s="38">
         <f t="shared" si="3"/>
         <v>15.073854388204486</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>12</v>
       </c>
@@ -3089,9 +3135,9 @@
         <v>30</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="D52" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="D52" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E52" s="2">
@@ -3113,12 +3159,12 @@
       <c r="J52" s="17">
         <v>5</v>
       </c>
-      <c r="K52" s="35">
+      <c r="K52" s="38">
         <f t="shared" si="3"/>
         <v>8.7035531239860209</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
@@ -3126,9 +3172,9 @@
         <v>30</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D53" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="D53" s="33" t="s">
         <v>15</v>
       </c>
       <c r="E53" s="2">
@@ -3150,19 +3196,261 @@
       <c r="J53" s="17">
         <v>5</v>
       </c>
-      <c r="K53" s="35">
+      <c r="K53" s="38">
         <f t="shared" si="3"/>
         <v>4.472091234310839</v>
       </c>
     </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="C54" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="D54" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="E54" s="31"/>
+      <c r="F54" s="31">
+        <v>500</v>
+      </c>
+      <c r="G54" s="32"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J54">
+        <v>5</v>
+      </c>
+      <c r="K54" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D55" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2">
+        <v>500</v>
+      </c>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J55">
+        <v>5</v>
+      </c>
+      <c r="K55" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D56" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2">
+        <v>500</v>
+      </c>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J56">
+        <v>5</v>
+      </c>
+      <c r="K56" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2">
+        <v>500</v>
+      </c>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J57">
+        <v>5</v>
+      </c>
+      <c r="K57" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B58" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2">
+        <v>500</v>
+      </c>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J58">
+        <v>5</v>
+      </c>
+      <c r="K58" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B59" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2">
+        <v>500</v>
+      </c>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J59">
+        <v>5</v>
+      </c>
+      <c r="K59" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B60" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D60" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2">
+        <v>500</v>
+      </c>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+      <c r="I60" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J60">
+        <v>5</v>
+      </c>
+      <c r="K60" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B61" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D61" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2">
+        <v>500</v>
+      </c>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="17">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="J61">
+        <v>5</v>
+      </c>
+      <c r="K61" s="38">
+        <f t="shared" si="3"/>
+        <v>4.472091234310839</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L53" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="N/A"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L61" xr:uid="{5B065B42-72D4-46A7-8F68-0B3E084D5031}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Aptos"&amp;10&amp;K000000 Interno&amp;1#_x000D_</oddHeader>
@@ -3188,15 +3476,15 @@
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -3204,7 +3492,7 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D6">
         <v>6</v>
@@ -3212,7 +3500,7 @@
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -3220,7 +3508,7 @@
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -3228,7 +3516,7 @@
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -3236,7 +3524,7 @@
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D10">
         <v>6</v>
@@ -3244,7 +3532,7 @@
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D11" s="5">
         <f>SUM(D5:D10)</f>
@@ -3253,25 +3541,25 @@
     </row>
     <row r="12" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C12">
         <v>10</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E12" s="6">
         <f>(D11*C12-C21)</f>
         <v>268</v>
       </c>
       <c r="I12" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D13" s="5" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="E13" s="6">
         <f>(E12*2)</f>
@@ -3280,7 +3568,7 @@
     </row>
     <row r="14" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="D14" s="5" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E14" s="6">
         <f>(E13*3)</f>
@@ -3289,13 +3577,13 @@
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="C17" s="10">
         <v>1</v>
@@ -3303,7 +3591,7 @@
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C18" s="10">
         <v>6</v>
@@ -3311,7 +3599,7 @@
     </row>
     <row r="19" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C19" s="10">
         <v>4</v>
@@ -3319,7 +3607,7 @@
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C20" s="10">
         <v>1</v>
@@ -3334,12 +3622,12 @@
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -3353,6 +3641,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="898695ca-150f-4d53-a1a4-27c213b72f41">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="11e3fce6-e222-4248-a00d-b3b33ed830c1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010023E2413248AD144EB4F352681303D788" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e915d9c603a07a4fc4694295454b5583">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="898695ca-150f-4d53-a1a4-27c213b72f41" xmlns:ns3="11e3fce6-e222-4248-a00d-b3b33ed830c1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b1e7ba0d6315b4b8ad6fa6ed50b7c17a" ns2:_="" ns3:_="">
     <xsd:import namespace="898695ca-150f-4d53-a1a4-27c213b72f41"/>
@@ -3547,27 +3855,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0855675D-7A7E-4EB6-A046-05A9ACCF1C10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="898695ca-150f-4d53-a1a4-27c213b72f41">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="11e3fce6-e222-4248-a00d-b3b33ed830c1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94EFCDE8-B628-4468-B13F-930C6557CB2F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="898695ca-150f-4d53-a1a4-27c213b72f41"/>
+    <ds:schemaRef ds:uri="11e3fce6-e222-4248-a00d-b3b33ed830c1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{591A5FB6-33BD-4B1F-88D8-436DAE7CA680}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3584,29 +3897,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0855675D-7A7E-4EB6-A046-05A9ACCF1C10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94EFCDE8-B628-4468-B13F-930C6557CB2F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="11e3fce6-e222-4248-a00d-b3b33ed830c1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="898695ca-150f-4d53-a1a4-27c213b72f41"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>